<commit_message>
scan: seg6 2026-08-10 15:53 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq7_2026-08-10.xlsx
+++ b/output/full_scan/batch_seq7_2026-08-10.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O80"/>
+  <dimension ref="A1:O76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -538,7 +538,7 @@
         <v/>
       </c>
       <c r="D2" s="2" t="n">
-        <v>759.8912550996769</v>
+        <v>719.8912550996769</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>1195</v>
@@ -591,7 +591,7 @@
         <v/>
       </c>
       <c r="D3" s="2" t="n">
-        <v>657.5891083167379</v>
+        <v>697.5891083167379</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>83.5</v>
@@ -644,7 +644,7 @@
         <v/>
       </c>
       <c r="D4" s="2" t="n">
-        <v>643.1425714737663</v>
+        <v>683.1425714737663</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>2845</v>
@@ -697,7 +697,7 @@
         <v/>
       </c>
       <c r="D5" s="2" t="n">
-        <v>639.0725445667794</v>
+        <v>679.0725445667794</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>145.5</v>
@@ -739,21 +739,21 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>6530</v>
+        <v>6642</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>創威</t>
+          <t>富致</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
         <v/>
       </c>
       <c r="D6" s="2" t="n">
-        <v>592.5901958258647</v>
+        <v>628.6846060253871</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>82.5</v>
+        <v>83.3</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -764,13 +764,13 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>55.3255704569258</v>
+        <v>60.2889815494212</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>23.70751846741007</v>
+        <v>17.20897975546421</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>1.819285779096404</v>
+        <v>4.284213476239731</v>
       </c>
       <c r="K6" s="2" t="n">
         <v>1</v>
@@ -782,31 +782,31 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>2.232003913636197</v>
+        <v>1.156990142525024</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, breakout_volume_confirm, cci_momentum, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, obv_uptrend, bb_squeeze_breakout, breakout_volume_confirm, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>6642</v>
+        <v>6530</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>富致</t>
+          <t>創威</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
         <v/>
       </c>
       <c r="D7" s="2" t="n">
-        <v>588.6846060253871</v>
+        <v>612.5901958258647</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>83.3</v>
+        <v>82.5</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
@@ -817,13 +817,13 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>60.2889815494212</v>
+        <v>55.3255704569258</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>17.20897975546421</v>
+        <v>23.70751846741007</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>4.284213476239731</v>
+        <v>1.819285779096404</v>
       </c>
       <c r="K7" s="2" t="n">
         <v>1</v>
@@ -835,31 +835,31 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>1.156990142525024</v>
+        <v>2.232003913636197</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, obv_uptrend, bb_squeeze_breakout, breakout_volume_confirm, mfi_strong</t>
+          <t>volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, breakout_volume_confirm, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>6789</v>
+        <v>6570</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>采鈺</t>
+          <t>維田</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
         <v/>
       </c>
       <c r="D8" s="2" t="n">
-        <v>580.558020671125</v>
+        <v>584.5426196577403</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>441.5</v>
+        <v>57.3</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -870,13 +870,13 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>45.60821881364068</v>
+        <v>62.78642047667233</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>22.20721067968122</v>
+        <v>17.51839189660703</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>0.8306212272732345</v>
+        <v>2.821798166333596</v>
       </c>
       <c r="K8" s="2" t="n">
         <v>0</v>
@@ -888,31 +888,31 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.7751631651231854</v>
+        <v>1.020147977210087</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, hist_turn_positive, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>6716</v>
+        <v>6651</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>應廣</t>
+          <t>全宇昕</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
         <v/>
       </c>
       <c r="D9" s="2" t="n">
-        <v>568.8507934837611</v>
+        <v>569.8512544222294</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>105</v>
+        <v>135</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -923,13 +923,13 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>66.65619037802345</v>
+        <v>55.2073267495169</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>21.99245011801612</v>
+        <v>21.67273944619703</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>1.408137471200302</v>
+        <v>2.739427404341888</v>
       </c>
       <c r="K9" s="2" t="n">
         <v>0</v>
@@ -941,31 +941,31 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>2.825541977084809</v>
+        <v>2.065680453017155</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, adx_trending, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>6672</v>
+        <v>6789</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>騰輝電子-KY</t>
+          <t>采鈺</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
         <v/>
       </c>
       <c r="D10" s="2" t="n">
-        <v>559.6551418881993</v>
+        <v>540.558020671125</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>251.5</v>
+        <v>441.5</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -976,13 +976,13 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>56.67183179011068</v>
+        <v>45.60821881364068</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>22.66951128365132</v>
+        <v>22.20721067968122</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>2.069419210418419</v>
+        <v>0.8306212272732345</v>
       </c>
       <c r="K10" s="2" t="n">
         <v>0</v>
@@ -994,48 +994,48 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>3.476117446306505</v>
+        <v>0.7751631651231854</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, hist_turn_positive, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>6669</v>
+        <v>6806</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>緯穎</t>
+          <t>森崴能源</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
         <v/>
       </c>
       <c r="D11" s="2" t="n">
-        <v>551.6128318963862</v>
+        <v>528.7768356926886</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>6010</v>
+        <v>3.51</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="G11" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>60.0720042164613</v>
+        <v>31.69502831466412</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>19.81404541536655</v>
+        <v>32.5931975692691</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>0.8392590884643881</v>
+        <v>2.013053626871306</v>
       </c>
       <c r="K11" s="2" t="n">
         <v>0</v>
@@ -1047,31 +1047,31 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>78.62252026483554</v>
+        <v>0.4112821443334762</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>6570</v>
+        <v>6672</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>維田</t>
+          <t>騰輝電子-KY</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
         <v/>
       </c>
       <c r="D12" s="2" t="n">
-        <v>544.5426196577403</v>
+        <v>519.6551418881993</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>57.3</v>
+        <v>251.5</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -1082,13 +1082,13 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>62.78642047667233</v>
+        <v>56.67183179011068</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>17.51839189660703</v>
+        <v>22.66951128365132</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>2.821798166333596</v>
+        <v>2.069419210418419</v>
       </c>
       <c r="K12" s="2" t="n">
         <v>0</v>
@@ -1100,31 +1100,31 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>1.020147977210087</v>
+        <v>3.476117446306505</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>6651</v>
+        <v>6669</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>全宇昕</t>
+          <t>緯穎</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
         <v/>
       </c>
       <c r="D13" s="2" t="n">
-        <v>529.8512544222294</v>
+        <v>511.6128318963861</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>135</v>
+        <v>6010</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -1135,13 +1135,13 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>55.2073267495169</v>
+        <v>60.0720042164613</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>21.67273944619703</v>
+        <v>19.81404541536655</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>2.739427404341888</v>
+        <v>0.8392590884643881</v>
       </c>
       <c r="K13" s="2" t="n">
         <v>0</v>
@@ -1153,48 +1153,48 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>2.065680453017155</v>
+        <v>78.62252026483554</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>6806</v>
+        <v>6640</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>森崴能源</t>
+          <t>均華</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
         <v/>
       </c>
       <c r="D14" s="2" t="n">
-        <v>528.7768356926886</v>
+        <v>485.7200540579751</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>3.51</v>
+        <v>1005</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G14" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>31.69502831466412</v>
+        <v>54.59927404791888</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>32.5931975692691</v>
+        <v>20.21834003709472</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>2.013053626871306</v>
+        <v>0.2956184699271068</v>
       </c>
       <c r="K14" s="2" t="n">
         <v>0</v>
@@ -1206,31 +1206,31 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0.4112821443334762</v>
+        <v>20.53216758736876</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, dealer_buy_3d, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>6805</v>
+        <v>6584</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>富世達</t>
+          <t>南俊國際</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
         <v/>
       </c>
       <c r="D15" s="2" t="n">
-        <v>507.7563613200152</v>
+        <v>469.236949088452</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>1755</v>
+        <v>522</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1241,13 +1241,13 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>61.11310339296048</v>
+        <v>46.18266784822475</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>30.83188965682062</v>
+        <v>30.31428625478637</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>1.860807352615913</v>
+        <v>3.581754449205871</v>
       </c>
       <c r="K15" s="2" t="n">
         <v>0</v>
@@ -1259,31 +1259,31 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>58.4128392384233</v>
+        <v>7.870487465498378</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>6830</v>
+        <v>6742</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>汎銓</t>
+          <t>澤米</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
         <v/>
       </c>
       <c r="D16" s="2" t="n">
-        <v>493.4382362107434</v>
+        <v>468.4734612140247</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>424.5</v>
+        <v>44.1</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -1294,13 +1294,13 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>52.54861417169353</v>
+        <v>40.82155755577556</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>21.29932834693594</v>
+        <v>21.68416843291506</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>1.119607925823429</v>
+        <v>0.3084014009874118</v>
       </c>
       <c r="K16" s="2" t="n">
         <v>0</v>
@@ -1312,31 +1312,31 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>15.16503674177781</v>
+        <v>0.5583314277996085</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>6533</v>
+        <v>6805</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>晶心科</t>
+          <t>富世達</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
         <v/>
       </c>
       <c r="D17" s="2" t="n">
-        <v>487.4846734611374</v>
+        <v>467.7563613200151</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>250</v>
+        <v>1755</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1347,13 +1347,13 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>63.32615909617144</v>
+        <v>61.11310339296048</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>17.84670684157508</v>
+        <v>30.83188965682062</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>3.13588276451926</v>
+        <v>1.860807352615913</v>
       </c>
       <c r="K17" s="2" t="n">
         <v>0</v>
@@ -1365,31 +1365,31 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>3.770773791979233</v>
+        <v>58.4128392384233</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>6743</v>
+        <v>6715</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>安普新</t>
+          <t>嘉基</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
         <v/>
       </c>
       <c r="D18" s="2" t="n">
-        <v>477.5575186325199</v>
+        <v>463.4202825676861</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>25.95</v>
+        <v>363.5</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -1400,13 +1400,13 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>33.87861410110625</v>
+        <v>47.29255753055375</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>30.65643176615675</v>
+        <v>11.21529419691228</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>0.8234789719637171</v>
+        <v>0.4688925881836271</v>
       </c>
       <c r="K18" s="2" t="n">
         <v>0</v>
@@ -1418,31 +1418,31 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>-0.5587045831037137</v>
+        <v>1.714932397652252</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, liquidity_ok, hist_turn_positive, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>6834</v>
+        <v>6830</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>天二科技</t>
+          <t>汎銓</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
         <v/>
       </c>
       <c r="D19" s="2" t="n">
-        <v>473.5071841860943</v>
+        <v>453.4382362107434</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>96.59999999999999</v>
+        <v>424.5</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -1453,13 +1453,13 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>51.42995958715492</v>
+        <v>52.54861417169353</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>18.11742300721276</v>
+        <v>21.29932834693594</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>1.088022397359117</v>
+        <v>1.119607925823429</v>
       </c>
       <c r="K19" s="2" t="n">
         <v>0</v>
@@ -1471,31 +1471,31 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>0.2480144407518252</v>
+        <v>15.16503674177781</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, liquidity_ok, hist_turn_positive, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>6640</v>
+        <v>6533</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>均華</t>
+          <t>晶心科</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
         <v/>
       </c>
       <c r="D20" s="2" t="n">
-        <v>465.7200540579751</v>
+        <v>447.4846734611374</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>1005</v>
+        <v>250</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -1506,13 +1506,13 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>54.59927404791888</v>
+        <v>63.32615909617144</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>20.21834003709472</v>
+        <v>17.84670684157508</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>0.2956184699271068</v>
+        <v>3.13588276451926</v>
       </c>
       <c r="K20" s="2" t="n">
         <v>0</v>
@@ -1524,31 +1524,31 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>20.53216758736876</v>
+        <v>3.770773791979233</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, dealer_buy_3d, cci_momentum, mfi_strong</t>
+          <t>volume_break, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>6715</v>
+        <v>6743</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>嘉基</t>
+          <t>安普新</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
         <v/>
       </c>
       <c r="D21" s="2" t="n">
-        <v>463.4202825676861</v>
+        <v>437.5575186325199</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>363.5</v>
+        <v>25.95</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1559,13 +1559,13 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>47.29255753055375</v>
+        <v>33.87861410110625</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>11.21529419691228</v>
+        <v>30.65643176615675</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>0.4688925881836271</v>
+        <v>0.8234789719637171</v>
       </c>
       <c r="K21" s="2" t="n">
         <v>0</v>
@@ -1577,31 +1577,31 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>1.714932397652252</v>
+        <v>-0.5587045831037137</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, liquidity_ok, hist_turn_positive, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>6756</v>
+        <v>6561</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>威鋒電子</t>
+          <t>是方</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
         <v/>
       </c>
       <c r="D22" s="2" t="n">
-        <v>447.6224378131971</v>
+        <v>433.7076490833803</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>99.90000000000001</v>
+        <v>327.5</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -1612,16 +1612,16 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>54.80601789098797</v>
+        <v>49.0884234657758</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>18.41246145425619</v>
+        <v>16.62347082415516</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>0.6046125239328692</v>
+        <v>0.5880489855703774</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L22" s="2" t="n">
         <v>0</v>
@@ -1630,31 +1630,31 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>1.074441310961462</v>
+        <v>1.208785345212072</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>6689</v>
+        <v>6834</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>伊雲谷</t>
+          <t>天二科技</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
         <v/>
       </c>
       <c r="D23" s="2" t="n">
-        <v>443.2327605734614</v>
+        <v>433.5071841860943</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>64.09999999999999</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
@@ -1665,13 +1665,13 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>58.1748589731627</v>
+        <v>51.42995958715492</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>24.78905494688414</v>
+        <v>18.11742300721276</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>1.359868348421285</v>
+        <v>1.088022397359117</v>
       </c>
       <c r="K23" s="2" t="n">
         <v>0</v>
@@ -1683,31 +1683,31 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0.6793548770186604</v>
+        <v>0.2480144407518252</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, liquidity_ok, hist_turn_positive, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>6742</v>
+        <v>6680</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>澤米</t>
+          <t>鑫創電子</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>438.4734612140247</v>
+        <v>432.1101223172679</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>44.1</v>
+        <v>52.9</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -1718,16 +1718,16 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>40.82155755577556</v>
+        <v>51.35654851602799</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>21.68416843291506</v>
+        <v>8.928063920683451</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>0.3084014009874118</v>
+        <v>0.8490717286048675</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L24" s="2" t="n">
         <v>0</v>
@@ -1736,31 +1736,31 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0.5583314277996085</v>
+        <v>-1.648866142513686</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, williams_r_recovery, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>6684</v>
+        <v>6689</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>安格</t>
+          <t>伊雲谷</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>436.0049317990572</v>
+        <v>423.2327605734614</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>50.2</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1771,16 +1771,16 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>51.55659956406806</v>
+        <v>58.1748589731627</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>16.81503294795015</v>
+        <v>24.78905494688414</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>1.238054269529925</v>
+        <v>1.359868348421285</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L25" s="2" t="n">
         <v>0</v>
@@ -1789,31 +1789,31 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0.1866763663144728</v>
+        <v>0.6793548770186604</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, hist_turn_positive, foreign_buy_3d, obv_uptrend</t>
+          <t>rsi_strong, market_above_ma60, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>6584</v>
+        <v>6756</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>南俊國際</t>
+          <t>威鋒電子</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>429.236949088452</v>
+        <v>407.6224378131971</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>522</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -1824,13 +1824,13 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>46.18266784822475</v>
+        <v>54.80601789098797</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>30.31428625478637</v>
+        <v>18.41246145425619</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>3.581754449205871</v>
+        <v>0.6046125239328692</v>
       </c>
       <c r="K26" s="2" t="n">
         <v>0</v>
@@ -1842,31 +1842,31 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>7.870487465498378</v>
+        <v>1.074441310961462</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>6658</v>
+        <v>6517</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>聯策</t>
+          <t>保勝光學</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>422.8295496624563</v>
+        <v>402.9592611202101</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>161.5</v>
+        <v>62</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -1877,16 +1877,16 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>49.57803870758161</v>
+        <v>43.65105831595943</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>23.76831546778813</v>
+        <v>17.74264075525872</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>0.7615987252108752</v>
+        <v>0.1284796058816047</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L27" s="2" t="n">
         <v>0</v>
@@ -1895,31 +1895,31 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>2.208044636336305</v>
+        <v>-0.4950825195650075</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>6691</v>
+        <v>6494</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>洋基工程</t>
+          <t>九齊</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>421.3977196089454</v>
+        <v>402.5202926201114</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>732</v>
+        <v>55.2</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1930,16 +1930,16 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>56.39326079237441</v>
+        <v>54.1229302849265</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>16.12405063835193</v>
+        <v>27.54430289878499</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>0.7817796276097244</v>
+        <v>1.14580192141777</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L28" s="2" t="n">
         <v>0</v>
@@ -1948,31 +1948,31 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>6.3943927806036</v>
+        <v>0.9095012201500574</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>6680</v>
+        <v>6658</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>鑫創電子</t>
+          <t>聯策</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>412.1101223172679</v>
+        <v>382.8295496624563</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>52.9</v>
+        <v>161.5</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1983,16 +1983,16 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>51.35654851602799</v>
+        <v>49.57803870758161</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>8.928063920683451</v>
+        <v>23.76831546778813</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>0.8490717286048675</v>
+        <v>0.7615987252108752</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L29" s="2" t="n">
         <v>0</v>
@@ -2001,31 +2001,31 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>-1.648866142513686</v>
+        <v>2.208044636336305</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, williams_r_recovery, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>6693</v>
+        <v>6691</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>廣閎科</t>
+          <t>洋基工程</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v/>
       </c>
       <c r="D30" s="2" t="n">
-        <v>409.4159036416215</v>
+        <v>381.3977196089454</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>184</v>
+        <v>732</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -2036,13 +2036,13 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>50.38863430194367</v>
+        <v>56.39326079237441</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>26.94908635017923</v>
+        <v>16.12405063835193</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>3.328927515200341</v>
+        <v>0.7817796276097244</v>
       </c>
       <c r="K30" s="2" t="n">
         <v>0</v>
@@ -2054,31 +2054,31 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>1.716256404857681</v>
+        <v>6.3943927806036</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>6561</v>
+        <v>6679</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>是方</t>
+          <t>鈺太</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>393.7076490833803</v>
+        <v>369.2154689917006</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>327.5</v>
+        <v>215.5</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -2089,16 +2089,16 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>49.0884234657758</v>
+        <v>43.50356665864479</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>16.62347082415516</v>
+        <v>31.37443742697766</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>0.5880489855703774</v>
+        <v>0.7293921328468287</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L31" s="2" t="n">
         <v>0</v>
@@ -2107,31 +2107,31 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>1.208785345212072</v>
+        <v>2.322547877028937</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>6517</v>
+        <v>6591</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>保勝光學</t>
+          <t>動力-KY</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>382.9592611202101</v>
+        <v>357.2464052793781</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>62</v>
+        <v>44.9</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -2142,16 +2142,16 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>43.65105831595943</v>
+        <v>42.13820941058614</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>17.74264075525872</v>
+        <v>45.03423550294112</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>0.1284796058816047</v>
+        <v>1.143389778792955</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L32" s="2" t="n">
         <v>0</v>
@@ -2160,31 +2160,31 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-0.4950825195650075</v>
+        <v>0.4851264654756431</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>6831</v>
+        <v>6664</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>邁科</t>
+          <t>群翊</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>367.7859982476213</v>
+        <v>348.442314200225</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>619</v>
+        <v>348</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -2195,16 +2195,16 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>47.22838285476606</v>
+        <v>47.45542651341767</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>23.85039667755416</v>
+        <v>25.70798519345708</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>0.92311151391005</v>
+        <v>0.7454550082529414</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L33" s="2" t="n">
         <v>0</v>
@@ -2213,31 +2213,31 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>9.930812126126725</v>
+        <v>1.261714691823794</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>6494</v>
+        <v>6556</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>九齊</t>
+          <t>勝品</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>362.5202926201114</v>
+        <v>341</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>55.2</v>
+        <v>61.7</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -2248,16 +2248,16 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>54.1229302849265</v>
+        <v>34.5926465168049</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>27.54430289878499</v>
+        <v>24.57604318797957</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>1.14580192141777</v>
+        <v>8.973581920851069</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L34" s="2" t="n">
         <v>0</v>
@@ -2266,31 +2266,31 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>0.9095012201500574</v>
+        <v>0.1846656717517687</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>6770</v>
+        <v>6548</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>力積電</t>
+          <t>長科*</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>354.947886614597</v>
+        <v>336.6128649838843</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>67.59999999999999</v>
+        <v>75.7</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -2301,16 +2301,16 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>53.55467541253191</v>
+        <v>53.05372729290665</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>16.20563895511379</v>
+        <v>19.98922929557009</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>1.169070819550472</v>
+        <v>0.6025674412759904</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L35" s="2" t="n">
         <v>0</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>1.266537678945586</v>
+        <v>1.19829039312493</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2340,7 +2340,7 @@
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>354.0242334417147</v>
+        <v>334.0242334417147</v>
       </c>
       <c r="E36" s="2" t="n">
         <v>88</v>
@@ -2382,21 +2382,21 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>6526</v>
+        <v>6588</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>達發</t>
+          <t>東典光電</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>353.9320709299399</v>
+        <v>329.377052895135</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>627</v>
+        <v>90.5</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2407,16 +2407,16 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>54.46587496093099</v>
+        <v>52.17663244556365</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>18.71173356855546</v>
+        <v>19.66415085566471</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>0.5119133710669493</v>
+        <v>0.4659584938125662</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L37" s="2" t="n">
         <v>0</v>
@@ -2425,31 +2425,31 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>12.25517051224604</v>
+        <v>1.975970167190084</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>6679</v>
+        <v>6831</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>鈺太</t>
+          <t>邁科</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v/>
       </c>
       <c r="D38" s="2" t="n">
-        <v>349.2154689917006</v>
+        <v>327.7859982476213</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>215.5</v>
+        <v>619</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2460,13 +2460,13 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>43.50356665864479</v>
+        <v>47.22838285476606</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>31.37443742697766</v>
+        <v>23.85039667755416</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>0.7293921328468287</v>
+        <v>0.92311151391005</v>
       </c>
       <c r="K38" s="2" t="n">
         <v>0</v>
@@ -2478,31 +2478,31 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>2.322547877028937</v>
+        <v>9.930812126126725</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>6708</v>
+        <v>6719</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>天擎</t>
+          <t>力智</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>347.7426857563657</v>
+        <v>325.9158525771313</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>38.8</v>
+        <v>205.5</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2513,13 +2513,13 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>51.82418142691544</v>
+        <v>40.82978142623313</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>13.21736218561355</v>
+        <v>20.79154253108725</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>0.3136627576445495</v>
+        <v>1.026644398199289</v>
       </c>
       <c r="K39" s="2" t="n">
         <v>0</v>
@@ -2531,31 +2531,31 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>0.6951912532277955</v>
+        <v>-0.1702043061906515</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, hist_turn_positive, obv_uptrend, williams_r_recovery, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>6641</v>
+        <v>6577</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>基士德-KY</t>
+          <t>勁豐</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>344.6382874993881</v>
+        <v>323.5857798095538</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>18.2</v>
+        <v>80.3</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2566,16 +2566,16 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>56.43482678571636</v>
+        <v>51.31890801893034</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>12.00180458616351</v>
+        <v>23.16408226615743</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>0.1768953973291743</v>
+        <v>0.1266768507117398</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L40" s="2" t="n">
         <v>0</v>
@@ -2584,31 +2584,31 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0.083393593295577</v>
+        <v>-0.3933678215734115</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, cci_momentum, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>6525</v>
+        <v>6770</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>捷敏-KY</t>
+          <t>力積電</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
         <v/>
       </c>
       <c r="D41" s="2" t="n">
-        <v>342.9680112976309</v>
+        <v>314.947886614597</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>142</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2619,13 +2619,13 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>48.54244158966806</v>
+        <v>53.55467541253191</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>22.13916893059711</v>
+        <v>16.20563895511379</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>0.5780713410641339</v>
+        <v>1.169070819550472</v>
       </c>
       <c r="K41" s="2" t="n">
         <v>0</v>
@@ -2637,31 +2637,31 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>-0.6126071199251202</v>
+        <v>1.266537678945586</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>6579</v>
+        <v>6526</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>研揚</t>
+          <t>達發</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>337.1238093422038</v>
+        <v>313.9320709299399</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>164.5</v>
+        <v>627</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2672,13 +2672,13 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>49.98277258133356</v>
+        <v>54.46587496093099</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>14.21627861852767</v>
+        <v>18.71173356855546</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>1.464210850067146</v>
+        <v>0.5119133710669493</v>
       </c>
       <c r="K42" s="2" t="n">
         <v>0</v>
@@ -2690,11 +2690,11 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>0.4912583213197818</v>
+        <v>12.25517051224604</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
@@ -2711,7 +2711,7 @@
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>336.7794053218618</v>
+        <v>306.7794053218618</v>
       </c>
       <c r="E43" s="2" t="n">
         <v>20.15</v>
@@ -2753,21 +2753,21 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>6591</v>
+        <v>6641</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>動力-KY</t>
+          <t>基士德-KY</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>327.2464052793781</v>
+        <v>304.6382874993881</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>44.9</v>
+        <v>18.2</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2778,13 +2778,13 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>42.13820941058614</v>
+        <v>56.43482678571636</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>45.03423550294112</v>
+        <v>12.00180458616351</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>1.143389778792955</v>
+        <v>0.1768953973291743</v>
       </c>
       <c r="K44" s="2" t="n">
         <v>0</v>
@@ -2796,31 +2796,31 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.4851264654756431</v>
+        <v>0.083393593295577</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>6719</v>
+        <v>6525</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>力智</t>
+          <t>捷敏-KY</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>325.9158525771313</v>
+        <v>302.9680112976309</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>205.5</v>
+        <v>142</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2831,13 +2831,13 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>40.82978142623313</v>
+        <v>48.54244158966806</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>20.79154253108725</v>
+        <v>22.13916893059711</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>1.026644398199289</v>
+        <v>0.5780713410641339</v>
       </c>
       <c r="K45" s="2" t="n">
         <v>0</v>
@@ -2849,31 +2849,31 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-0.1702043061906515</v>
+        <v>-0.6126071199251202</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>6556</v>
+        <v>6579</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>勝品</t>
+          <t>研揚</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>321</v>
+        <v>297.1238093422038</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>61.7</v>
+        <v>164.5</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2884,13 +2884,13 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>34.5926465168049</v>
+        <v>49.98277258133356</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>24.57604318797957</v>
+        <v>14.21627861852767</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>8.973581920851069</v>
+        <v>1.464210850067146</v>
       </c>
       <c r="K46" s="2" t="n">
         <v>0</v>
@@ -2902,11 +2902,11 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.1846656717517687</v>
+        <v>0.4912583213197818</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
@@ -2923,7 +2923,7 @@
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>311.7637366865634</v>
+        <v>291.7637366865634</v>
       </c>
       <c r="E47" s="2" t="n">
         <v>31</v>
@@ -2965,21 +2965,21 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>6664</v>
+        <v>6722</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>群翊</t>
+          <t>輝創</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>308.442314200225</v>
+        <v>290.4601890576815</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>348</v>
+        <v>33.25</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,16 +2990,16 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>47.45542651341767</v>
+        <v>41.43794222196013</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>25.70798519345708</v>
+        <v>45.09035858844592</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>0.7454550082529414</v>
+        <v>0.6582239260824728</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L48" s="2" t="n">
         <v>0</v>
@@ -3008,31 +3008,31 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>1.261714691823794</v>
+        <v>0.0453051647860042</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>6577</v>
+        <v>6683</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>勁豐</t>
+          <t>雍智科技</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>303.5857798095538</v>
+        <v>286.538427429983</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>80.3</v>
+        <v>1230</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,16 +3043,16 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>51.31890801893034</v>
+        <v>48.2745948886829</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>23.16408226615743</v>
+        <v>28.25725879420688</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>0.1266768507117398</v>
+        <v>0.4899732956481283</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L49" s="2" t="n">
         <v>0</v>
@@ -3061,31 +3061,31 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-0.3933678215734115</v>
+        <v>31.4348537002561</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>6548</v>
+        <v>6531</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>長科*</t>
+          <t>愛普*</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>296.6128649838843</v>
+        <v>284.7992152405097</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>75.7</v>
+        <v>923</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,16 +3096,16 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>53.05372729290665</v>
+        <v>55.53775567986045</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>19.98922929557009</v>
+        <v>17.9383876361415</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0.6025674412759904</v>
+        <v>1.776806020075897</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L50" s="2" t="n">
         <v>0</v>
@@ -3114,31 +3114,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>1.19829039312493</v>
+        <v>26.79131172666612</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>6588</v>
+        <v>6613</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>東典光電</t>
+          <t>朋億*</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>289.377052895135</v>
+        <v>278.7082956743713</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>90.5</v>
+        <v>267</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,16 +3149,16 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>52.17663244556365</v>
+        <v>39.02089114142221</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>19.66415085566471</v>
+        <v>17.92466641318843</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.4659584938125662</v>
+        <v>1.295821904755391</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L51" s="2" t="n">
         <v>0</v>
@@ -3167,31 +3167,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>1.975970167190084</v>
+        <v>-2.564751388353312</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>6581</v>
+        <v>6546</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>鋼聯</t>
+          <t>正基</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>288.2253586697184</v>
+        <v>276.6720293204235</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>108</v>
+        <v>61.1</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,16 +3202,16 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>49.67379398493452</v>
+        <v>48.6918563128969</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>13.01856406597112</v>
+        <v>34.25128176075999</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.3520176135133184</v>
+        <v>0.4540382745166306</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L52" s="2" t="n">
         <v>0</v>
@@ -3220,31 +3220,31 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.0219361556607685</v>
+        <v>0.8710308901620962</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>6515</v>
+        <v>6568</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>穎崴</t>
+          <t>宏觀</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>281.0314674116885</v>
+        <v>253.4327049767064</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>6830</v>
+        <v>139.5</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,16 +3255,16 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>48.71305714719616</v>
+        <v>44.11459787240925</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>19.23198677474299</v>
+        <v>50.3952196306465</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.9790195446006202</v>
+        <v>0.5120552148809838</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L53" s="2" t="n">
         <v>0</v>
@@ -3273,31 +3273,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>181.6138323572908</v>
+        <v>2.265521062470729</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, kd_golden_cross</t>
+          <t>market_above_ma60, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>6546</v>
+        <v>6667</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>正基</t>
+          <t>信紘科</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>276.6720293204235</v>
+        <v>252.4384138177306</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>61.1</v>
+        <v>235.5</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,16 +3308,16 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>48.6918563128969</v>
+        <v>45.71064707908463</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>34.25128176075999</v>
+        <v>26.92820647933205</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.4540382745166306</v>
+        <v>0.8239079445400816</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L54" s="2" t="n">
         <v>0</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.8710308901620962</v>
+        <v>1.098253347595543</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>6692</v>
+        <v>6581</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>進能服</t>
+          <t>鋼聯</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>274.8501039559089</v>
+        <v>248.2253586697184</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>24.25</v>
+        <v>108</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,16 +3361,16 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>52.26106510648049</v>
+        <v>49.67379398493452</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>11.43825607522764</v>
+        <v>13.01856406597112</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>3.244331776378185</v>
+        <v>0.3520176135133184</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L55" s="2" t="n">
         <v>0</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.5307021697131324</v>
+        <v>0.0219361556607685</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>6722</v>
+        <v>6515</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>輝創</t>
+          <t>穎崴</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>260.4601890576815</v>
+        <v>241.0314674116884</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>33.25</v>
+        <v>6830</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,13 +3414,13 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>41.43794222196013</v>
+        <v>48.71305714719616</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>45.09035858844592</v>
+        <v>19.23198677474299</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.6582239260824728</v>
+        <v>0.9790195446006202</v>
       </c>
       <c r="K56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.0453051647860042</v>
+        <v>181.6138323572908</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>6667</v>
+        <v>6698</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>信紘科</t>
+          <t>旭暉應材</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>252.4384138177306</v>
+        <v>235.1009942776442</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>235.5</v>
+        <v>34.05</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,13 +3467,13 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>45.71064707908463</v>
+        <v>44.76379528547555</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>26.92820647933205</v>
+        <v>23.3107845556375</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.8239079445400816</v>
+        <v>0.5893334830166511</v>
       </c>
       <c r="K57" s="2" t="n">
         <v>0</v>
@@ -3485,31 +3485,31 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>1.098253347595543</v>
+        <v>0.2970275502286945</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>6683</v>
+        <v>6488</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>雍智科技</t>
+          <t>環球晶</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>246.538427429983</v>
+        <v>226.296324417609</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>1230</v>
+        <v>854</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,49 +3520,49 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>48.2745948886829</v>
+        <v>40.00740011950307</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>28.25725879420688</v>
+        <v>19.6361494784886</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>0.4899732956481283</v>
+        <v>0.6090360424699359</v>
       </c>
       <c r="K58" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L58" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M58" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>31.4348537002561</v>
+        <v>-27.16885309080623</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>6597</v>
+        <v>6654</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>立誠</t>
+          <t>天正國際</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>245.8405061488688</v>
+        <v>224.6346304023602</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>67.8</v>
+        <v>175.5</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,13 +3573,13 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>52.56550927441516</v>
+        <v>52.30623216854402</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>9.227910220942441</v>
+        <v>20.35072611833792</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>2.222963075213416</v>
+        <v>0.5443752742378344</v>
       </c>
       <c r="K59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>1.657113472402883</v>
+        <v>0.8049146976001036</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>6776</v>
+        <v>6695</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>展碁國際</t>
+          <t>芯鼎</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>239.3388245766569</v>
+        <v>223.9700088630154</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>54</v>
+        <v>49.05</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,13 +3626,13 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>47.18497562275842</v>
+        <v>42.38783163284979</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>21.12908600125668</v>
+        <v>16.84054063700665</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.6309677549372419</v>
+        <v>0.5859369776776999</v>
       </c>
       <c r="K60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.1513933882284058</v>
+        <v>-0.04727762318667</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>6613</v>
+        <v>6597</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>朋億*</t>
+          <t>立誠</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>238.7082956743713</v>
+        <v>215.8405061488688</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>267</v>
+        <v>67.8</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,13 +3679,13 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>39.02089114142221</v>
+        <v>52.56550927441516</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>17.92466641318843</v>
+        <v>9.227910220942441</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>1.295821904755391</v>
+        <v>2.222963075213416</v>
       </c>
       <c r="K61" s="2" t="n">
         <v>0</v>
@@ -3697,31 +3697,31 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-2.564751388353312</v>
+        <v>1.657113472402883</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>volume_break, market_above_ma60, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>6488</v>
+        <v>6674</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>環球晶</t>
+          <t>鋐寶科技</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>226.296324417609</v>
+        <v>211.4543449681333</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>854</v>
+        <v>15.15</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,49 +3732,49 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>40.00740011950307</v>
+        <v>33.09777697734876</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>19.6361494784886</v>
+        <v>27.94371380273006</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0.6090360424699359</v>
+        <v>1.233427896138704</v>
       </c>
       <c r="K62" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L62" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M62" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-27.16885309080623</v>
+        <v>-0.0109324870091924</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>6568</v>
+        <v>6485</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>宏觀</t>
+          <t>點序</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>213.4327049767064</v>
+        <v>210.1515967327581</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>139.5</v>
+        <v>65.2</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,13 +3785,13 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>44.11459787240925</v>
+        <v>46.58153637139367</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>50.3952196306465</v>
+        <v>31.92566440614958</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0.5120552148809838</v>
+        <v>0.8886209377032902</v>
       </c>
       <c r="K63" s="2" t="n">
         <v>1</v>
@@ -3803,31 +3803,31 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>2.265521062470729</v>
+        <v>1.451334781405931</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>6624</v>
+        <v>6560</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>萬年清</t>
+          <t>欣普羅</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>212.9192891707028</v>
+        <v>208.2895459900261</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>43.55</v>
+        <v>32.75</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,13 +3838,13 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>54.1956178298716</v>
+        <v>42.6656646377571</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>10.31840855293046</v>
+        <v>23.55610304861302</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0.0808055944507439</v>
+        <v>0.09574777521272169</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0</v>
@@ -3856,31 +3856,31 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>3.456389985290163</v>
+        <v>0.2164267139628419</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>6485</v>
+        <v>6486</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>點序</t>
+          <t>互動</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>210.1515967327581</v>
+        <v>205.11694768226</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>65.2</v>
+        <v>74.8</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,16 +3891,16 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>46.58153637139367</v>
+        <v>37.32295600264841</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>31.92566440614958</v>
+        <v>20.93066759831938</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.8886209377032902</v>
+        <v>0.4384345853634585</v>
       </c>
       <c r="K65" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L65" s="2" t="n">
         <v>0</v>
@@ -3909,31 +3909,31 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>1.451334781405931</v>
+        <v>-0.0291627746541869</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>6668</v>
+        <v>6776</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>中揚光</t>
+          <t>展碁國際</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>206.9074690674686</v>
+        <v>199.3388245766569</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>35.25</v>
+        <v>54</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3944,13 +3944,13 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>47.20786546979786</v>
+        <v>47.18497562275842</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>14.09140970435063</v>
+        <v>21.12908600125668</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.3209328948822644</v>
+        <v>0.6309677549372419</v>
       </c>
       <c r="K66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.1986078361931164</v>
+        <v>0.1513933882284058</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>6698</v>
+        <v>6706</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>旭暉應材</t>
+          <t>惠特</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>205.1009942776442</v>
+        <v>195.4078662588853</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>34.05</v>
+        <v>115</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,13 +3997,13 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>44.76379528547555</v>
+        <v>47.36422328239001</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>23.3107845556375</v>
+        <v>27.9360274930259</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.5893334830166511</v>
+        <v>1.400283400510497</v>
       </c>
       <c r="K67" s="2" t="n">
         <v>0</v>
@@ -4015,31 +4015,31 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.2970275502286945</v>
+        <v>3.154285057340575</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>6792</v>
+        <v>6668</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>詠業</t>
+          <t>中揚光</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>201.4577717824017</v>
+        <v>186.9074690674686</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>58.1</v>
+        <v>35.25</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4050,13 +4050,13 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>53.53094301456269</v>
+        <v>47.20786546979786</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>20.83237706136118</v>
+        <v>14.09140970435063</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>0.1071657777679421</v>
+        <v>0.3209328948822644</v>
       </c>
       <c r="K68" s="2" t="n">
         <v>0</v>
@@ -4068,31 +4068,31 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>0.9151082857450872</v>
+        <v>0.1986078361931164</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending, cci_momentum</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>6695</v>
+        <v>6624</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>芯鼎</t>
+          <t>萬年清</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>193.9700088630154</v>
+        <v>182.9192891707028</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>49.05</v>
+        <v>43.55</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4103,13 +4103,13 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>42.38783163284979</v>
+        <v>54.1956178298716</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>16.84054063700665</v>
+        <v>10.31840855293046</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.5859369776776999</v>
+        <v>0.0808055944507439</v>
       </c>
       <c r="K69" s="2" t="n">
         <v>0</v>
@@ -4121,31 +4121,31 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-0.04727762318667</v>
+        <v>3.456389985290163</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>6643</v>
+        <v>6792</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>M31</t>
+          <t>詠業</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>188.3184728606389</v>
+        <v>181.4577717824017</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>441</v>
+        <v>58.1</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,16 +4156,16 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>51.4404446531714</v>
+        <v>53.53094301456269</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>16.8644077092416</v>
+        <v>20.83237706136118</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.6067073503653335</v>
+        <v>0.1071657777679421</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L70" s="2" t="n">
         <v>0</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>7.946861437298072</v>
+        <v>0.9151082857450872</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, mfi_strong</t>
+          <t>market_above_ma60, adx_trending, cci_momentum</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>6654</v>
+        <v>6552</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>天正國際</t>
+          <t>易華電</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>184.6346304023602</v>
+        <v>168.5981297540415</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>175.5</v>
+        <v>24.9</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,13 +4209,13 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>52.30623216854402</v>
+        <v>42.38434697611292</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>20.35072611833792</v>
+        <v>22.7585018338222</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.5443752742378344</v>
+        <v>0.259430816537764</v>
       </c>
       <c r="K71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.8049146976001036</v>
+        <v>0.191439221867006</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>6573</v>
+        <v>6498</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>虹揚-KY</t>
+          <t>久禾光</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>183.1716928791651</v>
+        <v>166.1113844479647</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>16.95</v>
+        <v>77</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,13 +4262,13 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>42.60033215073253</v>
+        <v>43.16491929246962</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>16.91018142212874</v>
+        <v>38.13070991314</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.5594342595761482</v>
+        <v>0.8679145084146477</v>
       </c>
       <c r="K72" s="2" t="n">
         <v>0</v>
@@ -4280,31 +4280,31 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.2575969118523213</v>
+        <v>0.8198042544683419</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>6674</v>
+        <v>6573</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>鋐寶科技</t>
+          <t>虹揚-KY</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>181.4543449681333</v>
+        <v>163.1716928791651</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>15.15</v>
+        <v>16.95</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -4315,13 +4315,13 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>33.09777697734876</v>
+        <v>42.60033215073253</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>27.94371380273006</v>
+        <v>16.91018142212874</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>1.233427896138704</v>
+        <v>0.5594342595761482</v>
       </c>
       <c r="K73" s="2" t="n">
         <v>0</v>
@@ -4333,31 +4333,31 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-0.0109324870091924</v>
+        <v>-0.2575969118523213</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>6558</v>
+        <v>6643</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>興能高</t>
+          <t>M31</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>172.9799379394085</v>
+        <v>158.3184728606389</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>26.75</v>
+        <v>441</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,16 +4368,16 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>49.35985312135943</v>
+        <v>51.4404446531714</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>31.78033287105508</v>
+        <v>16.8644077092416</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.9041300013487308</v>
+        <v>0.6067073503653335</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L74" s="2" t="n">
         <v>0</v>
@@ -4386,31 +4386,31 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.2548989916106241</v>
+        <v>7.946861437298072</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending</t>
+          <t>market_above_ma60, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>6560</v>
+        <v>6771</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>欣普羅</t>
+          <t>平和環保-創</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>168.2895459900261</v>
+        <v>142.8745263239954</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>32.75</v>
+        <v>38</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,13 +4421,13 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>42.6656646377571</v>
+        <v>39.90102792412294</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>23.55610304861302</v>
+        <v>13.84143715119434</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.09574777521272169</v>
+        <v>1.307740811853606</v>
       </c>
       <c r="K75" s="2" t="n">
         <v>0</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>0.2164267139628419</v>
+        <v>0.07260361763226519</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>6706</v>
+        <v>6558</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>惠特</t>
+          <t>興能高</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>165.4078662588853</v>
+        <v>132.9799379394085</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>115</v>
+        <v>26.75</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,13 +4474,13 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>47.36422328239001</v>
+        <v>49.35985312135943</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>27.9360274930259</v>
+        <v>31.78033287105508</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>1.400283400510497</v>
+        <v>0.9041300013487308</v>
       </c>
       <c r="K76" s="2" t="n">
         <v>0</v>
@@ -4492,223 +4492,11 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>3.154285057340575</v>
+        <v>0.2548989916106241</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, adx_trending</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="2" t="n">
-        <v>6486</v>
-      </c>
-      <c r="B77" s="2" t="inlineStr">
-        <is>
-          <t>互動</t>
-        </is>
-      </c>
-      <c r="C77" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D77" s="2" t="n">
-        <v>165.11694768226</v>
-      </c>
-      <c r="E77" s="2" t="n">
-        <v>74.8</v>
-      </c>
-      <c r="F77" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="G77" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H77" s="2" t="n">
-        <v>37.32295600264841</v>
-      </c>
-      <c r="I77" s="2" t="n">
-        <v>20.93066759831938</v>
-      </c>
-      <c r="J77" s="2" t="n">
-        <v>0.4384345853634585</v>
-      </c>
-      <c r="K77" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L77" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M77" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N77" s="2" t="n">
-        <v>-0.0291627746541869</v>
-      </c>
-      <c r="O77" s="2" t="inlineStr">
-        <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="2" t="n">
-        <v>6498</v>
-      </c>
-      <c r="B78" s="2" t="inlineStr">
-        <is>
-          <t>久禾光</t>
-        </is>
-      </c>
-      <c r="C78" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D78" s="2" t="n">
-        <v>146.1113844479647</v>
-      </c>
-      <c r="E78" s="2" t="n">
-        <v>77</v>
-      </c>
-      <c r="F78" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="G78" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H78" s="2" t="n">
-        <v>43.16491929246962</v>
-      </c>
-      <c r="I78" s="2" t="n">
-        <v>38.13070991314</v>
-      </c>
-      <c r="J78" s="2" t="n">
-        <v>0.8679145084146477</v>
-      </c>
-      <c r="K78" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L78" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M78" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N78" s="2" t="n">
-        <v>0.8198042544683419</v>
-      </c>
-      <c r="O78" s="2" t="inlineStr">
-        <is>
           <t>market_above_ma60, adx_trending</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="2" t="n">
-        <v>6552</v>
-      </c>
-      <c r="B79" s="2" t="inlineStr">
-        <is>
-          <t>易華電</t>
-        </is>
-      </c>
-      <c r="C79" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D79" s="2" t="n">
-        <v>138.5981297540415</v>
-      </c>
-      <c r="E79" s="2" t="n">
-        <v>24.9</v>
-      </c>
-      <c r="F79" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="G79" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H79" s="2" t="n">
-        <v>42.38434697611292</v>
-      </c>
-      <c r="I79" s="2" t="n">
-        <v>22.7585018338222</v>
-      </c>
-      <c r="J79" s="2" t="n">
-        <v>0.259430816537764</v>
-      </c>
-      <c r="K79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M79" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N79" s="2" t="n">
-        <v>0.191439221867006</v>
-      </c>
-      <c r="O79" s="2" t="inlineStr">
-        <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="2" t="n">
-        <v>6771</v>
-      </c>
-      <c r="B80" s="2" t="inlineStr">
-        <is>
-          <t>平和環保-創</t>
-        </is>
-      </c>
-      <c r="C80" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D80" s="2" t="n">
-        <v>112.8745263239954</v>
-      </c>
-      <c r="E80" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="F80" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="G80" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H80" s="2" t="n">
-        <v>39.90102792412294</v>
-      </c>
-      <c r="I80" s="2" t="n">
-        <v>13.84143715119434</v>
-      </c>
-      <c r="J80" s="2" t="n">
-        <v>1.307740811853606</v>
-      </c>
-      <c r="K80" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L80" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M80" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N80" s="2" t="n">
-        <v>0.07260361763226519</v>
-      </c>
-      <c r="O80" s="2" t="inlineStr">
-        <is>
-          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>

</xml_diff>